<commit_message>
Fix spell descriptions and image matching
</commit_message>
<xml_diff>
--- a/Dungeon Master/Viko/Paladin Spells.xlsx
+++ b/Dungeon Master/Viko/Paladin Spells.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604e5eff5508ce9/Desktop/WIZARD SPELLS/Viko/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604e5eff5508ce9/Desktop/WIZARD SPELLS/Dungeon Master/Viko/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="192" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA9C28BB-223F-4B60-A1D1-C4C2BFE6D99B}"/>
+  <xr:revisionPtr revIDLastSave="193" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2A9A181-6B8B-4B17-A413-5DA4516CB099}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3624" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{1A773363-9EAE-4410-83FA-4C280E3FC519}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{1A773363-9EAE-4410-83FA-4C280E3FC519}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1579,6 +1579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M43"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1710,7 +1711,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
         <v>1</v>
       </c>
@@ -1776,7 +1777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>1</v>
       </c>
@@ -1809,7 +1810,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.600000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="18.600000000000001" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>1</v>
       </c>
@@ -1842,7 +1843,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>1</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -1908,7 +1909,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -1941,7 +1942,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>1</v>
       </c>
@@ -1974,7 +1975,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <v>1</v>
       </c>
@@ -2005,7 +2006,7 @@
       </c>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <v>1</v>
       </c>
@@ -2038,7 +2039,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <v>1</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>1</v>
       </c>
@@ -2137,7 +2138,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>1</v>
       </c>
@@ -2203,7 +2204,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <v>2</v>
       </c>
@@ -2269,7 +2270,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="22" t="s">
@@ -2300,7 +2301,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <v>2</v>
       </c>
@@ -2366,7 +2367,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" ht="24" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <v>2</v>
       </c>
@@ -2399,7 +2400,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" ht="27" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <v>2</v>
       </c>
@@ -2432,7 +2433,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <v>2</v>
       </c>
@@ -2465,7 +2466,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <v>2</v>
       </c>
@@ -2498,7 +2499,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="18" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <v>2</v>
       </c>
@@ -2531,7 +2532,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <v>2</v>
       </c>
@@ -2798,7 +2799,13 @@
       <c r="B43"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K36" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}"/>
+  <autoFilter ref="A1:K36" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="SI"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Potencialmente">
       <formula>NOT(ISERROR(SEARCH("Potencialmente",E1)))</formula>

</xml_diff>

<commit_message>
Añadir tipo de hechizo por tarjeta, niveles de personaje, creación de hechizos y sincronización online
</commit_message>
<xml_diff>
--- a/Dungeon Master/Viko/Paladin Spells.xlsx
+++ b/Dungeon Master/Viko/Paladin Spells.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604e5eff5508ce9/Desktop/WIZARD SPELLS/Dungeon Master/Viko/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="193" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2A9A181-6B8B-4B17-A413-5DA4516CB099}"/>
+  <xr:revisionPtr revIDLastSave="210" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA3B9BE-6776-44C4-84FE-EFA596ABF5D1}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{1A773363-9EAE-4410-83FA-4C280E3FC519}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$K$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$L$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
     <author>jonathan mendoza</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{32951713-9D17-403A-A465-1C06D758C1A9}">
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{32951713-9D17-403A-A465-1C06D758C1A9}">
       <text>
         <r>
           <rPr>
@@ -71,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{842802F5-0B70-43B6-B6B9-6AF5B1E3E170}">
+    <comment ref="E4" authorId="0" shapeId="0" xr:uid="{842802F5-0B70-43B6-B6B9-6AF5B1E3E170}">
       <text>
         <r>
           <rPr>
@@ -95,7 +95,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{407995EA-1329-476D-856B-FF1E6EEB40D6}">
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{407995EA-1329-476D-856B-FF1E6EEB40D6}">
       <text>
         <r>
           <rPr>
@@ -125,7 +125,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{EC04B6F8-8974-46B2-9B54-3DFF62CC3D11}">
+    <comment ref="E9" authorId="0" shapeId="0" xr:uid="{EC04B6F8-8974-46B2-9B54-3DFF62CC3D11}">
       <text>
         <r>
           <rPr>
@@ -159,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{C698BA4B-E60F-46B8-ABB5-C173F7A02B2F}">
+    <comment ref="E11" authorId="0" shapeId="0" xr:uid="{C698BA4B-E60F-46B8-ABB5-C173F7A02B2F}">
       <text>
         <r>
           <rPr>
@@ -189,7 +189,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{385D89A3-5A98-46C0-BC92-D938C26B1213}">
+    <comment ref="E16" authorId="0" shapeId="0" xr:uid="{385D89A3-5A98-46C0-BC92-D938C26B1213}">
       <text>
         <r>
           <rPr>
@@ -215,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{14A51346-6B65-482E-8FB2-0999667508BC}">
+    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{14A51346-6B65-482E-8FB2-0999667508BC}">
       <text>
         <r>
           <rPr>
@@ -239,7 +239,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{A75A82D0-95F8-4297-9FB1-B6E773D298EF}">
+    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{A75A82D0-95F8-4297-9FB1-B6E773D298EF}">
       <text>
         <r>
           <rPr>
@@ -267,7 +267,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{9D340120-FD9B-45A8-B703-DE2CDD4CE69D}">
+    <comment ref="E29" authorId="0" shapeId="0" xr:uid="{9D340120-FD9B-45A8-B703-DE2CDD4CE69D}">
       <text>
         <r>
           <rPr>
@@ -295,7 +295,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{625B758A-DC89-4380-9420-ADDE11DF2156}">
+    <comment ref="E32" authorId="0" shapeId="0" xr:uid="{625B758A-DC89-4380-9420-ADDE11DF2156}">
       <text>
         <r>
           <rPr>
@@ -333,7 +333,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{EF62F056-7573-4A3B-AADB-09CF052CAA05}">
+    <comment ref="E35" authorId="0" shapeId="0" xr:uid="{EF62F056-7573-4A3B-AADB-09CF052CAA05}">
       <text>
         <r>
           <rPr>
@@ -390,7 +390,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="160">
   <si>
     <t>NIVEL</t>
   </si>
@@ -888,6 +888,12 @@
   </si>
   <si>
     <t>https://drive.google.com/uc?export=view&amp;id=1unqHFj53iWIzdPGqzdPf5pk9SA-CyT5n</t>
+  </si>
+  <si>
+    <t>Efecto</t>
+  </si>
+  <si>
+    <t>Daño</t>
   </si>
 </sst>
 </file>
@@ -1579,26 +1585,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="3"/>
     <col min="2" max="2" width="54" style="3" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" customWidth="1"/>
-    <col min="4" max="4" width="35.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.88671875" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="48.21875" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="71.77734375" hidden="1" customWidth="1"/>
+    <col min="3" max="4" width="27.33203125" customWidth="1"/>
+    <col min="5" max="5" width="35.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.88671875" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="48.21875" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="71.77734375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1606,75 +1611,81 @@
       <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="26"/>
+      <c r="N1" s="26" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="214.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="214.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="9" t="e" vm="1">
-        <f>IF(M2="","",_xlfn.IMAGE(M2,"",0))</f>
+        <f>IF(N2="","",_xlfn.IMAGE(N2,"",0))</f>
         <v>#VALUE!</v>
       </c>
       <c r="C2" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="I2" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="J2" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="K2" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="M2" s="27" t="s">
+      <c r="N2" s="27" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1682,36 +1693,39 @@
       <c r="C3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="G3" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="I3" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="L3" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="L3" t="str">
-        <f>IF(M3="","",_xlfn.IMAGE(M3,"",0))</f>
+      <c r="M3" t="str">
+        <f>IF(N3="","",_xlfn.IMAGE(N3,"",0))</f>
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1719,32 +1733,35 @@
       <c r="C4" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K4" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
         <v>1</v>
       </c>
@@ -1752,32 +1769,35 @@
       <c r="C5" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="F5" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="H5" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="I5" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J5" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K5" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>1</v>
       </c>
@@ -1785,32 +1805,35 @@
       <c r="C6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I6" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J6" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.600000000000001" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="18.600000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>1</v>
       </c>
@@ -1818,32 +1841,35 @@
       <c r="C7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>53</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J7" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>1</v>
       </c>
@@ -1851,32 +1877,35 @@
       <c r="C8" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="F8" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="G8" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="H8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="I8" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -1884,32 +1913,35 @@
       <c r="C9" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E9" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="G9" s="12" t="s">
         <v>133</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K9" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L9" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -1917,32 +1949,35 @@
       <c r="C10" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="G10" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="I10" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="J10" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J10" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L10" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>1</v>
       </c>
@@ -1950,32 +1985,35 @@
       <c r="C11" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="F11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="G11" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="J11" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J11" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <v>1</v>
       </c>
@@ -1983,30 +2021,33 @@
       <c r="C12" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="G12" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="H12" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="I12" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="K12" s="10"/>
-    </row>
-    <row r="13" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L12" s="10"/>
+    </row>
+    <row r="13" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <v>1</v>
       </c>
@@ -2014,32 +2055,35 @@
       <c r="C13" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="G13" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="I13" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="I13" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J13" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K13" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L13" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <v>1</v>
       </c>
@@ -2047,32 +2091,35 @@
       <c r="C14" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="G14" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="H14" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="I14" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="J14" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J14" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K14" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L14" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>1</v>
       </c>
@@ -2080,32 +2127,35 @@
       <c r="C15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="G15" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="I15" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="J15" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J15" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K15" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L15" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <v>1</v>
       </c>
@@ -2113,32 +2163,35 @@
       <c r="C16" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="E16" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="G16" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="I16" s="10" t="s">
         <v>71</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>96</v>
       </c>
       <c r="K16" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L16" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>1</v>
       </c>
@@ -2146,32 +2199,35 @@
       <c r="C17" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="F17" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="G17" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="I17" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J17" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K17" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L17" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <v>2</v>
       </c>
@@ -2179,32 +2235,35 @@
       <c r="C18" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="G18" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="I18" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J18" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K18" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K18" s="10" t="s">
+      <c r="L18" s="10" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <v>2</v>
       </c>
@@ -2212,32 +2271,35 @@
       <c r="C19" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E19" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="H19" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="I19" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="J19" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J19" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K19" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L19" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <v>2</v>
       </c>
@@ -2245,63 +2307,69 @@
       <c r="C20" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="E20" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="F20" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="G20" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="H20" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="I20" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="I20" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J20" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K20" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="L20" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="F21" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="G21" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="H21" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="I21" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="J21" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J21" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K21" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L21" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <v>2</v>
       </c>
@@ -2309,32 +2377,35 @@
       <c r="C22" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E22" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="H22" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="I22" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I22" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J22" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K22" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L22" s="10" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <v>2</v>
       </c>
@@ -2342,32 +2413,35 @@
       <c r="C23" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E23" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="F23" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="G23" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="J23" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K23" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K23" s="10" t="s">
+      <c r="L23" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="24" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <v>2</v>
       </c>
@@ -2375,32 +2449,35 @@
       <c r="C24" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="F24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="G24" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="H24" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="I24" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="I24" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J24" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K24" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L24" s="10" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="27" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <v>2</v>
       </c>
@@ -2408,32 +2485,35 @@
       <c r="C25" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E25" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="F25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="G25" s="14" t="s">
         <v>55</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I25" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J25" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="J25" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="K25" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L25" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <v>2</v>
       </c>
@@ -2441,32 +2521,35 @@
       <c r="C26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="E26" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="F26" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="G26" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="H26" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="I26" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="I26" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J26" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K26" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L26" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <v>2</v>
       </c>
@@ -2474,32 +2557,35 @@
       <c r="C27" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="E27" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="F27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F27" s="12" t="s">
+      <c r="G27" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="H27" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="I27" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="I27" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J27" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K27" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L27" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="18" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <v>2</v>
       </c>
@@ -2507,32 +2593,35 @@
       <c r="C28" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E28" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="F28" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="13" t="s">
+      <c r="G28" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="H28" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="H28" s="10" t="s">
+      <c r="I28" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="I28" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J28" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K28" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L28" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <v>2</v>
       </c>
@@ -2540,30 +2629,33 @@
       <c r="C29" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="E29" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="F29" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F29" s="12" t="s">
+      <c r="G29" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="10" t="s">
+      <c r="H29" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10" t="s">
-        <v>54</v>
-      </c>
+      <c r="I29" s="10"/>
       <c r="J29" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K29" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L29" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
         <v>103</v>
       </c>
@@ -2571,32 +2663,35 @@
       <c r="C30" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="E30" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="F30" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F30" s="12" t="s">
+      <c r="G30" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="H30" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="I30" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="I30" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J30" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K30" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K30" s="10" t="s">
+      <c r="L30" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="16" t="s">
         <v>103</v>
       </c>
@@ -2604,32 +2699,35 @@
       <c r="C31" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E31" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="F31" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F31" s="12" t="s">
+      <c r="G31" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="H31" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="I31" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="J31" s="10" t="s">
         <v>96</v>
       </c>
       <c r="K31" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L31" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
         <v>103</v>
       </c>
@@ -2637,32 +2735,35 @@
       <c r="C32" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E32" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="F32" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F32" s="12" t="s">
+      <c r="G32" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="H32" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="I32" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="J32" s="10" t="s">
         <v>96</v>
       </c>
       <c r="K32" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L32" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>103</v>
       </c>
@@ -2670,32 +2771,35 @@
       <c r="C33" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E33" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="F33" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="G33" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="H33" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="I33" s="10" t="s">
         <v>71</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="J33" s="10" t="s">
         <v>96</v>
       </c>
       <c r="K33" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L33" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="20.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="20.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="17" t="s">
         <v>107</v>
       </c>
@@ -2703,32 +2807,35 @@
       <c r="C34" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="E34" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="F34" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F34" s="12" t="s">
+      <c r="G34" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="G34" s="12" t="s">
+      <c r="H34" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="I34" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I34" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J34" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K34" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K34" s="10" t="s">
+      <c r="L34" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="17" t="s">
         <v>107</v>
       </c>
@@ -2736,32 +2843,35 @@
       <c r="C35" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E35" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="F35" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F35" s="12" t="s">
+      <c r="G35" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="G35" s="10" t="s">
+      <c r="H35" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="I35" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="I35" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J35" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K35" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K35" s="10" t="s">
+      <c r="L35" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>107</v>
       </c>
@@ -2769,64 +2879,61 @@
       <c r="C36" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="E36" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="F36" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F36" s="10" t="s">
+      <c r="G36" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="H36" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="I36" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="I36" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="J36" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K36" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="K36" s="10" t="s">
+      <c r="L36" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B43"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K36" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="SI"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <conditionalFormatting sqref="E1:E1048576">
+  <autoFilter ref="A1:L36" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}"/>
+  <conditionalFormatting sqref="F1:F1048576">
     <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Potencialmente">
-      <formula>NOT(ISERROR(SEARCH("Potencialmente",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Potencialmente",F1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="No">
-      <formula>NOT(ISERROR(SEARCH("No",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("No",F1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Si">
-      <formula>NOT(ISERROR(SEARCH("Si",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Si",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:J1048576 K36:M36">
+  <conditionalFormatting sqref="J1:K1048576 L36:N36">
     <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="No">
-      <formula>NOT(ISERROR(SEARCH("No",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("No",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="Si">
-      <formula>NOT(ISERROR(SEARCH("Si",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Si",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="M2" r:id="rId1" xr:uid="{410E7E23-63A7-46F2-B06F-EB7BB7721689}"/>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{410E7E23-63A7-46F2-B06F-EB7BB7721689}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>